<commit_message>
data(page7 two-table caliber, user ruling): drop dual-high concept; objective line >=15 problem points (48 communities) + subjective line >=50 complaints ~= 1/week (47 communities); overlap exactly 10 communities (map-overlay target); integer depth tiers with weekly-frequency narrative; sync csv/Excel(4 sheets)/both data-package mds/RAG note + index rebuild
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATA/analysis/汇总/图数表出图_PPT表格汇总.xlsx
+++ b/DATA/analysis/汇总/图数表出图_PPT表格汇总.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2610" yWindow="0" windowWidth="28740" windowHeight="20985" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6000" yWindow="0" windowWidth="21930" windowHeight="20985" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="page1" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="2">
     <font>
       <name val="宋体"/>
       <family val="2"/>
@@ -30,81 +30,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <b val="1"/>
-      <i val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <name val="宋体"/>
       <charset val="134"/>
       <family val="3"/>
       <sz val="9"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <family val="2"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -115,118 +45,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF808080"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -236,243 +60,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF808080"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>

</xml_diff>